<commit_message>
refactor: rename milk category type from Cattle Milk to Cow Milk
</commit_message>
<xml_diff>
--- a/Farm_Expenses_And_Revenue_Tracker.xlsx
+++ b/Farm_Expenses_And_Revenue_Tracker.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="135">
   <si>
     <t>Expense ID</t>
   </si>
@@ -83,7 +83,7 @@
     <t>Veterinary Doctor</t>
   </si>
   <si>
-    <t>Cattle health checkup</t>
+    <t>Cow health checkup</t>
   </si>
   <si>
     <t>EXP-105</t>
@@ -98,9 +98,6 @@
     <t>EXP-106</t>
   </si>
   <si>
-    <t>Concentrate feed</t>
-  </si>
-  <si>
     <t>EXP-107</t>
   </si>
   <si>
@@ -110,7 +107,7 @@
     <t>EXP-108</t>
   </si>
   <si>
-    <t>Cattle Store</t>
+    <t>Cow Store</t>
   </si>
   <si>
     <t>Punnaku bag</t>
@@ -176,7 +173,7 @@
     <t>Dharshan</t>
   </si>
   <si>
-    <t>Cattle Milk</t>
+    <t>Cow Milk</t>
   </si>
   <si>
     <t>Daily Customer</t>
@@ -368,7 +365,7 @@
     <t>Bottle Size / Item</t>
   </si>
   <si>
-    <t>Cattle Milk Rate (Rs.)</t>
+    <t>Cow Milk Rate (Rs.)</t>
   </si>
   <si>
     <t>Goat Milk Rate (Rs.)</t>
@@ -1065,15 +1062,15 @@
         <v>450</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>12</v>
@@ -1090,42 +1087,42 @@
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E9" s="4">
         <v>500</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>34</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E10" s="4">
         <v>1200</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1152,66 +1149,66 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="C1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>49</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>56</v>
       </c>
       <c r="G2" s="3">
         <v>0</v>
@@ -1229,7 +1226,7 @@
         <v>1</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M2" s="6">
         <f>SUMIF('Daily Tracker'!D2:D100, B2, 'Daily Tracker'!J2:J100)</f>
@@ -1240,22 +1237,22 @@
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="G3" s="3">
         <v>10</v>
@@ -1273,7 +1270,7 @@
         <v>15</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M3" s="6">
         <f>SUMIF('Daily Tracker'!D2:D100, B3, 'Daily Tracker'!J2:J100)</f>
@@ -1284,22 +1281,22 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>67</v>
       </c>
       <c r="G4" s="3">
         <v>2</v>
@@ -1317,7 +1314,7 @@
         <v>0</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M4" s="6">
         <f>SUMIF('Daily Tracker'!D2:D100, B4, 'Daily Tracker'!J2:J100)</f>
@@ -1328,22 +1325,22 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="G5" s="3">
         <v>0</v>
@@ -1361,7 +1358,7 @@
         <v>25</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M5" s="6">
         <f>SUMIF('Daily Tracker'!D2:D100, B5, 'Daily Tracker'!J2:J100)</f>
@@ -1372,22 +1369,22 @@
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="E6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>75</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>76</v>
       </c>
       <c r="G6" s="3">
         <v>0</v>
@@ -1405,7 +1402,7 @@
         <v>0</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="M6" s="6">
         <f>SUMIF('Daily Tracker'!D2:D100, B6, 'Daily Tracker'!J2:J100)</f>
@@ -1445,84 +1442,84 @@
         <v>1</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>40</v>
-      </c>
       <c r="D1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="P1" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="Q1" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="P1" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="Q1" s="10" t="s">
+      <c r="R1" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="R1" s="10" t="s">
+      <c r="S1" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="T1" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="U1" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="U1" s="10" t="s">
+      <c r="V1" s="11" t="s">
         <v>93</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="W1" s="7" t="s">
         <v>94</v>
-      </c>
-      <c r="W1" s="7" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>97</v>
       </c>
       <c r="E2" s="12">
         <v>10</v>
@@ -1579,21 +1576,21 @@
         <f>P2-U2</f>
       </c>
       <c r="W2" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>99</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>100</v>
       </c>
       <c r="E3" s="12">
         <v>12</v>
@@ -1650,21 +1647,21 @@
         <f>P3-U3</f>
       </c>
       <c r="W3" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>102</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>103</v>
       </c>
       <c r="E4" s="12">
         <v>5</v>
@@ -1721,21 +1718,21 @@
         <f>P4-U4</f>
       </c>
       <c r="W4" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="D5" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E5" s="12">
         <v>8</v>
@@ -1792,21 +1789,21 @@
         <f>P5-U5</f>
       </c>
       <c r="W5" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E6" s="12">
         <v>15</v>
@@ -1863,21 +1860,21 @@
         <f>P6-U6</f>
       </c>
       <c r="W6" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="C7" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>109</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>110</v>
       </c>
       <c r="E7" s="13">
         <f>SUM(E2:E6)</f>
@@ -1934,7 +1931,7 @@
         <f>SUM(V2:V6)</f>
       </c>
       <c r="W7" s="13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1956,7 +1953,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -1964,27 +1961,27 @@
     </row>
     <row r="2" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B2" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="D2" s="18" t="s">
         <v>114</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B3" s="6">
-        <f>SUMIF('Daily Tracker'!B2:B6, "Cattle Milk", 'Daily Tracker'!J2:J6)</f>
+        <f>SUMIF('Daily Tracker'!B2:B6, "Cow Milk", 'Daily Tracker'!J2:J6)</f>
       </c>
       <c r="C3" s="4">
-        <f>SUMIF('Daily Tracker'!B2:B6, "Cattle Milk", 'Daily Tracker'!P2:P6)</f>
+        <f>SUMIF('Daily Tracker'!B2:B6, "Cow Milk", 'Daily Tracker'!P2:P6)</f>
       </c>
       <c r="D3" s="19">
         <f>IF(C3&gt;0, C3/SUM($C$3:$C$4), 0)</f>
@@ -1992,7 +1989,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B4" s="6">
         <f>SUMIF('Daily Tracker'!B2:B6, "Goat Milk", 'Daily Tracker'!J2:J6)</f>
@@ -2025,24 +2022,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
+        <v>115</v>
+      </c>
+      <c r="B1" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="C1" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="D1" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="E1" s="20" t="s">
         <v>119</v>
-      </c>
-      <c r="E1" s="20" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B2" s="4">
         <v>15</v>
@@ -2051,15 +2048,15 @@
         <v>25</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B3" s="4">
         <v>35</v>
@@ -2068,15 +2065,15 @@
         <v>60</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>125</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B4" s="4">
         <v>38</v>
@@ -2085,15 +2082,15 @@
         <v>65</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>128</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B5" s="4">
         <v>50</v>
@@ -2102,15 +2099,15 @@
         <v>90</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>131</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B6" s="4">
         <v>65</v>
@@ -2119,10 +2116,10 @@
         <v>120</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>134</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add Customer Master Excel generator & register 36 clean customers
</commit_message>
<xml_diff>
--- a/Farm_Expenses_And_Revenue_Tracker.xlsx
+++ b/Farm_Expenses_And_Revenue_Tracker.xlsx
@@ -9,13 +9,14 @@
     <sheet sheetId="3" name="Daily Tracker" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Milk Category Summary" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Rates &amp; Settings" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Customer Master" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="219">
   <si>
     <t>Expense ID</t>
   </si>
@@ -420,6 +421,258 @@
   </si>
   <si>
     <t>Editable: Unit price for 1000ml (1L) bottle</t>
+  </si>
+  <si>
+    <t>Payment Type</t>
+  </si>
+  <si>
+    <t>Milk Type</t>
+  </si>
+  <si>
+    <t>Delivery Address / Notes</t>
+  </si>
+  <si>
+    <t>Helabojun</t>
+  </si>
+  <si>
+    <t>Cow Milk Only</t>
+  </si>
+  <si>
+    <t>Route Sales / Spot</t>
+  </si>
+  <si>
+    <t>Goat Milk Sales</t>
+  </si>
+  <si>
+    <t>Goat Milk Only</t>
+  </si>
+  <si>
+    <t>Goat Milk Route</t>
+  </si>
+  <si>
+    <t>Ayurveda</t>
+  </si>
+  <si>
+    <t>Ayurveda Center</t>
+  </si>
+  <si>
+    <t>Gamini</t>
+  </si>
+  <si>
+    <t>Route Sales</t>
+  </si>
+  <si>
+    <t>Lakeside</t>
+  </si>
+  <si>
+    <t>Weekly Customer</t>
+  </si>
+  <si>
+    <t>Lakeside Area</t>
+  </si>
+  <si>
+    <t>CUST-106</t>
+  </si>
+  <si>
+    <t>Mahaiyyawa</t>
+  </si>
+  <si>
+    <t>Mahaiyyawa Route</t>
+  </si>
+  <si>
+    <t>CUST-107</t>
+  </si>
+  <si>
+    <t>Arupola Hotel</t>
+  </si>
+  <si>
+    <t>Arupola Route</t>
+  </si>
+  <si>
+    <t>CUST-108</t>
+  </si>
+  <si>
+    <t>Karthik</t>
+  </si>
+  <si>
+    <t>Town Route</t>
+  </si>
+  <si>
+    <t>CUST-109</t>
+  </si>
+  <si>
+    <t>Logeshwaran</t>
+  </si>
+  <si>
+    <t>Monthly Account</t>
+  </si>
+  <si>
+    <t>CUST-110</t>
+  </si>
+  <si>
+    <t>Praveen</t>
+  </si>
+  <si>
+    <t>CUST-111</t>
+  </si>
+  <si>
+    <t>Lekraj</t>
+  </si>
+  <si>
+    <t>CUST-112</t>
+  </si>
+  <si>
+    <t>Nursery</t>
+  </si>
+  <si>
+    <t>CUST-113</t>
+  </si>
+  <si>
+    <t>Mahendran</t>
+  </si>
+  <si>
+    <t>CUST-114</t>
+  </si>
+  <si>
+    <t>Ravi Ranjan Pandit</t>
+  </si>
+  <si>
+    <t>CUST-115</t>
+  </si>
+  <si>
+    <t>Wijesoriya</t>
+  </si>
+  <si>
+    <t>CUST-116</t>
+  </si>
+  <si>
+    <t>Vinayagamoorthy</t>
+  </si>
+  <si>
+    <t>CUST-117</t>
+  </si>
+  <si>
+    <t>Aadithya</t>
+  </si>
+  <si>
+    <t>CUST-118</t>
+  </si>
+  <si>
+    <t>Selvanayagi</t>
+  </si>
+  <si>
+    <t>CUST-119</t>
+  </si>
+  <si>
+    <t>Jeyachandrika</t>
+  </si>
+  <si>
+    <t>CUST-120</t>
+  </si>
+  <si>
+    <t>Safras</t>
+  </si>
+  <si>
+    <t>CUST-121</t>
+  </si>
+  <si>
+    <t>Yogesh</t>
+  </si>
+  <si>
+    <t>CUST-122</t>
+  </si>
+  <si>
+    <t>Uthpala Wickramasinghe</t>
+  </si>
+  <si>
+    <t>CUST-123</t>
+  </si>
+  <si>
+    <t>Sundar</t>
+  </si>
+  <si>
+    <t>CUST-124</t>
+  </si>
+  <si>
+    <t>Asgiriya</t>
+  </si>
+  <si>
+    <t>Asgiriya Route</t>
+  </si>
+  <si>
+    <t>CUST-125</t>
+  </si>
+  <si>
+    <t>Periya Samy (Dada)</t>
+  </si>
+  <si>
+    <t>CUST-126</t>
+  </si>
+  <si>
+    <t>Hardware</t>
+  </si>
+  <si>
+    <t>CUST-127</t>
+  </si>
+  <si>
+    <t>Ranga</t>
+  </si>
+  <si>
+    <t>CUST-128</t>
+  </si>
+  <si>
+    <t>Nithya</t>
+  </si>
+  <si>
+    <t>CUST-129</t>
+  </si>
+  <si>
+    <t>Pramod Sharma</t>
+  </si>
+  <si>
+    <t>CUST-130</t>
+  </si>
+  <si>
+    <t>Sathosa Thenna</t>
+  </si>
+  <si>
+    <t>CUST-131</t>
+  </si>
+  <si>
+    <t>Keerthana</t>
+  </si>
+  <si>
+    <t>CUST-132</t>
+  </si>
+  <si>
+    <t>Eb Ayya</t>
+  </si>
+  <si>
+    <t>CUST-133</t>
+  </si>
+  <si>
+    <t>Eb Akka</t>
+  </si>
+  <si>
+    <t>CUST-134</t>
+  </si>
+  <si>
+    <t>Pichamalwatta</t>
+  </si>
+  <si>
+    <t>Pichamalwatta Route</t>
+  </si>
+  <si>
+    <t>CUST-135</t>
+  </si>
+  <si>
+    <t>Vidhu</t>
+  </si>
+  <si>
+    <t>CUST-136</t>
+  </si>
+  <si>
+    <t>Ahiran</t>
   </si>
 </sst>
 </file>
@@ -2126,4 +2379,875 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Employee Registration and Salary/Payroll Management system
</commit_message>
<xml_diff>
--- a/Farm_Expenses_And_Revenue_Tracker.xlsx
+++ b/Farm_Expenses_And_Revenue_Tracker.xlsx
@@ -10,13 +10,14 @@
     <sheet sheetId="4" name="Milk Category Summary" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Rates &amp; Settings" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Customer Master" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Employee Master" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="241">
   <si>
     <t>Expense ID</t>
   </si>
@@ -673,6 +674,72 @@
   </si>
   <si>
     <t>Ahiran</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>Employee Name</t>
+  </si>
+  <si>
+    <t>Job Designation</t>
+  </si>
+  <si>
+    <t>Pay Structure</t>
+  </si>
+  <si>
+    <t>Base Rate / Salary (Rs.)</t>
+  </si>
+  <si>
+    <t>Joined Date</t>
+  </si>
+  <si>
+    <t>EMP-101</t>
+  </si>
+  <si>
+    <t>Murugan Worker</t>
+  </si>
+  <si>
+    <t>Grass Cutter &amp; Laborer</t>
+  </si>
+  <si>
+    <t>0771234567</t>
+  </si>
+  <si>
+    <t>Daily Wage</t>
+  </si>
+  <si>
+    <t>2026-01-15</t>
+  </si>
+  <si>
+    <t>EMP-102</t>
+  </si>
+  <si>
+    <t>Farm Herdsman</t>
+  </si>
+  <si>
+    <t>0779876543</t>
+  </si>
+  <si>
+    <t>Monthly Salary</t>
+  </si>
+  <si>
+    <t>2026-02-01</t>
+  </si>
+  <si>
+    <t>EMP-103</t>
+  </si>
+  <si>
+    <t>Ravi</t>
+  </si>
+  <si>
+    <t>Milker &amp; Farm Worker</t>
+  </si>
+  <si>
+    <t>0751122334</t>
+  </si>
+  <si>
+    <t>2026-03-10</t>
   </si>
 </sst>
 </file>
@@ -3250,4 +3317,128 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
+        <v>219</v>
+      </c>
+      <c r="B1" s="20" t="s">
+        <v>220</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="D1" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="F1" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="G1" s="20" t="s">
+        <v>224</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F2" s="4">
+        <v>600</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="F3" s="4">
+        <v>25000</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F4" s="4">
+        <v>750</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>